<commit_message>
St Pete monthly data
Monthly data pull. Quarterly data updates.
</commit_message>
<xml_diff>
--- a/Data/CERP_PBC_Summary_Data.xlsx
+++ b/Data/CERP_PBC_Summary_Data.xlsx
@@ -39494,6 +39494,286 @@
         <v>0</v>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="3" t="n">
+        <v>45870</v>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>45890</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>100</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="3" t="n">
+        <v>45890</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" t="n">
+        <v>100</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" s="3" t="n">
+        <v>45874</v>
+      </c>
+      <c r="M30" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" t="n">
+        <v>100</v>
+      </c>
+      <c r="P30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q30" s="3" t="n">
+        <v>45874</v>
+      </c>
+      <c r="R30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S30" t="n">
+        <v>0</v>
+      </c>
+      <c r="T30" t="n">
+        <v>93.33</v>
+      </c>
+      <c r="U30" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="V30" s="3" t="n">
+        <v>45874</v>
+      </c>
+      <c r="W30" t="n">
+        <v>0</v>
+      </c>
+      <c r="X30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y30" t="n">
+        <v>100</v>
+      </c>
+      <c r="Z30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA30" s="3" t="n">
+        <v>45874</v>
+      </c>
+      <c r="AB30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD30" t="n">
+        <v>100</v>
+      </c>
+      <c r="AE30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF30" s="3" t="n">
+        <v>45875</v>
+      </c>
+      <c r="AG30" t="n">
+        <v>7.14</v>
+      </c>
+      <c r="AH30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI30" t="n">
+        <v>85.71</v>
+      </c>
+      <c r="AJ30" t="n">
+        <v>7.14</v>
+      </c>
+      <c r="AK30" s="3" t="n">
+        <v>45875</v>
+      </c>
+      <c r="AL30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM30" t="n">
+        <v>7.14</v>
+      </c>
+      <c r="AN30" t="n">
+        <v>71.43</v>
+      </c>
+      <c r="AO30" t="n">
+        <v>21.43</v>
+      </c>
+      <c r="AP30" s="3" t="n">
+        <v>45875</v>
+      </c>
+      <c r="AQ30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS30" t="n">
+        <v>100</v>
+      </c>
+      <c r="AT30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="n">
+        <v>45901</v>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>45916</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
+        <v>100</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="3" t="n">
+        <v>45916</v>
+      </c>
+      <c r="H31" t="n">
+        <v>10</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" t="n">
+        <v>90</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" s="3" t="n">
+        <v>45902</v>
+      </c>
+      <c r="M31" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" t="n">
+        <v>100</v>
+      </c>
+      <c r="P31" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q31" s="3" t="n">
+        <v>45902</v>
+      </c>
+      <c r="R31" t="n">
+        <v>0</v>
+      </c>
+      <c r="S31" t="n">
+        <v>0</v>
+      </c>
+      <c r="T31" t="n">
+        <v>100</v>
+      </c>
+      <c r="U31" t="n">
+        <v>0</v>
+      </c>
+      <c r="V31" s="3" t="n">
+        <v>45903</v>
+      </c>
+      <c r="W31" t="n">
+        <v>7.14</v>
+      </c>
+      <c r="X31" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y31" t="n">
+        <v>85.71</v>
+      </c>
+      <c r="Z31" t="n">
+        <v>7.14</v>
+      </c>
+      <c r="AA31" s="3" t="n">
+        <v>45904</v>
+      </c>
+      <c r="AB31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD31" t="n">
+        <v>100</v>
+      </c>
+      <c r="AE31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF31" s="3" t="n">
+        <v>45903</v>
+      </c>
+      <c r="AG31" t="n">
+        <v>14.29</v>
+      </c>
+      <c r="AH31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI31" t="n">
+        <v>57.14</v>
+      </c>
+      <c r="AJ31" t="n">
+        <v>28.57</v>
+      </c>
+      <c r="AK31" s="3" t="n">
+        <v>45903</v>
+      </c>
+      <c r="AL31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN31" t="n">
+        <v>92.31</v>
+      </c>
+      <c r="AO31" t="n">
+        <v>7.69</v>
+      </c>
+      <c r="AP31" s="3" t="n">
+        <v>45903</v>
+      </c>
+      <c r="AQ31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS31" t="n">
+        <v>100</v>
+      </c>
+      <c r="AT31" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>